<commit_message>
Sxxx: Add Short text column (#2388)
* Sxxx: Add Short text column

* Fix
</commit_message>
<xml_diff>
--- a/java/bundles/org.eclipse.set.feature/rootdir/data/export/excel/sxxx_vorlage.xlsx
+++ b/java/bundles/org.eclipse.set.feature/rootdir/data/export/excel/sxxx_vorlage.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ws_intern\planpro\repos\set\java\bundles\org.eclipse.set.feature\rootdir\data\export\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ws_intern\planpro\set\java\bundles\org.eclipse.set.feature\rootdir\data\export\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6E9CD98-EFDE-4181-8ECC-8B101C39FFFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCC17B29-7251-4E95-8340-BA23433128AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="50820" windowHeight="20745" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sskz" sheetId="6" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sskz!$A$1:$C$52</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sskz!$A$1:$E$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Sskz!$1:$4</definedName>
   </definedNames>
   <calcPr calcId="145621"/>
@@ -24,16 +24,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>A</t>
   </si>
   <si>
     <t>B</t>
-  </si>
-  <si>
-    <t>Inhalt
-Bearbeitungsvermerk</t>
   </si>
   <si>
     <t>Referenziert von Objekt</t>
@@ -43,6 +39,18 @@
   </si>
   <si>
     <t>C</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>Kurztext</t>
+  </si>
+  <si>
+    <t>Bearbeitungsvermerk</t>
+  </si>
+  <si>
+    <t>Inhalt</t>
   </si>
 </sst>
 </file>
@@ -71,7 +79,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -155,11 +163,77 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -179,9 +253,6 @@
     <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -193,6 +264,24 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -522,13 +611,15 @@
       <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
@@ -567,14 +658,15 @@
       <c r="AO1" s="2"/>
     </row>
     <row r="2" spans="2:41" ht="37.700000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="12"/>
+      <c r="D2" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="E2" s="7" t="s">
         <v>3</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>4</v>
       </c>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
@@ -582,16 +674,21 @@
       <c r="J2" s="3"/>
     </row>
     <row r="3" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="3"/>
+      <c r="B3" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
       <c r="J3" s="3"/>
     </row>
     <row r="4" spans="2:41" ht="13.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="7"/>
-      <c r="C4" s="6"/>
+      <c r="B4" s="16"/>
+      <c r="C4" s="14"/>
       <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
     </row>
     <row r="5" spans="2:41" x14ac:dyDescent="0.25">
       <c r="B5" s="4"/>
@@ -602,6 +699,7 @@
     </row>
     <row r="6" spans="2:41" x14ac:dyDescent="0.25">
       <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
@@ -856,10 +954,8 @@
       <c r="G52" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
+  <mergeCells count="1">
+    <mergeCell ref="B2:C2"/>
   </mergeCells>
   <printOptions gridLines="1"/>
   <pageMargins left="0.78740157480314965" right="0.39370078740157483" top="0.19685039370078741" bottom="0.59055118110236227" header="0" footer="0"/>
@@ -868,77 +964,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_Version xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <_DCDateModified xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <_Status xmlns="http://schemas.microsoft.com/sharepoint/v3/fields">Nicht begonnen</_Status>
-    <_Revision xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <_DCDateCreated xmlns="http://schemas.microsoft.com/sharepoint/v3/fields"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<LongProperties xmlns="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100E758A0F93049BE4CAD441F10C0D8186D" ma:contentTypeVersion="5" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="fb340e34ecc5d059b634082484788e96">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="576ce185-3b2e-4f75-8b7c-efeb82226bea" xmlns:ns3="http://schemas.microsoft.com/sharepoint/v3/fields" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ae5cd419a40dc0c21009e0c04d2bd83e" ns2:_="" ns3:_="">
     <xsd:import namespace="576ce185-3b2e-4f75-8b7c-efeb82226bea"/>
@@ -1130,48 +1155,78 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<LongProperties xmlns="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
+</file>
+
+<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_Version xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <_DCDateModified xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <_Status xmlns="http://schemas.microsoft.com/sharepoint/v3/fields">Nicht begonnen</_Status>
+    <_Revision xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <_DCDateCreated xmlns="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1177B4BE-B106-4A5F-9B8B-849CAD24B948}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="576ce185-3b2e-4f75-8b7c-efeb82226bea"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5FA61470-DD61-4999-8627-225AC049B66F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{947F1741-2986-4B63-8B5C-D0468C671233}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A1C5838C-81AB-4B9A-B282-4E4B57DAFB8B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FD45C59E-C13E-4B92-9551-AE1790848EFA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1188,4 +1243,45 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A1C5838C-81AB-4B9A-B282-4E4B57DAFB8B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{947F1741-2986-4B63-8B5C-D0468C671233}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5FA61470-DD61-4999-8627-225AC049B66F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1177B4BE-B106-4A5F-9B8B-849CAD24B948}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="576ce185-3b2e-4f75-8b7c-efeb82226bea"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fix some export bugs (#2509)
* fix merging of cells in excel export

* use font of first cell in header as fallback

* fix print area of sxxx template

* extend table model by isRemarkColumn

* properly configure isRemarkColumn for all the tables

* improve utiltity function name and usage

* fix detection of remark columns in pdf exports

* fix duplicate footnote shorthands in excel export

* retrieve workbook from sheet

* explain font fallback

* make function abstract because overriden in almost all the places
</commit_message>
<xml_diff>
--- a/java/bundles/org.eclipse.set.feature/rootdir/data/export/excel/sxxx_vorlage.xlsx
+++ b/java/bundles/org.eclipse.set.feature/rootdir/data/export/excel/sxxx_vorlage.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ws_intern\planpro\set\java\bundles\org.eclipse.set.feature\rootdir\data\export\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ws_intern\planpro\repos\set\java\bundles\org.eclipse.set.feature\rootdir\data\export\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCC17B29-7251-4E95-8340-BA23433128AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DBFCAA7-3F9F-49AC-ACD9-F0CAADED5D8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="50850" windowHeight="20625" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sskz" sheetId="6" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sskz!$A$1:$E$6</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sskz!$A:$E</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Sskz!$1:$4</definedName>
   </definedNames>
   <calcPr calcId="145621"/>
@@ -233,7 +233,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -265,23 +265,26 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -658,10 +661,10 @@
       <c r="AO1" s="2"/>
     </row>
     <row r="2" spans="2:41" ht="37.700000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="12"/>
+      <c r="C2" s="16"/>
       <c r="D2" s="7" t="s">
         <v>2</v>
       </c>
@@ -674,10 +677,10 @@
       <c r="J2" s="3"/>
     </row>
     <row r="3" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="11" t="s">
         <v>8</v>
       </c>
       <c r="D3" s="8"/>
@@ -685,14 +688,16 @@
       <c r="J3" s="3"/>
     </row>
     <row r="4" spans="2:41" ht="13.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="16"/>
-      <c r="C4" s="14"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="12"/>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
     </row>
     <row r="5" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B5" s="4"/>
-      <c r="E5" s="4"/>
+      <c r="B5" s="17"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="17"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -964,6 +969,77 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_Version xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <_DCDateModified xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <_Status xmlns="http://schemas.microsoft.com/sharepoint/v3/fields">Nicht begonnen</_Status>
+    <_Revision xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <_DCDateCreated xmlns="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<LongProperties xmlns="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100E758A0F93049BE4CAD441F10C0D8186D" ma:contentTypeVersion="5" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="fb340e34ecc5d059b634082484788e96">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="576ce185-3b2e-4f75-8b7c-efeb82226bea" xmlns:ns3="http://schemas.microsoft.com/sharepoint/v3/fields" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ae5cd419a40dc0c21009e0c04d2bd83e" ns2:_="" ns3:_="">
     <xsd:import namespace="576ce185-3b2e-4f75-8b7c-efeb82226bea"/>
@@ -1155,78 +1231,48 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<LongProperties xmlns="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
-</file>
-
-<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_Version xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <_DCDateModified xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <_Status xmlns="http://schemas.microsoft.com/sharepoint/v3/fields">Nicht begonnen</_Status>
-    <_Revision xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <_DCDateCreated xmlns="http://schemas.microsoft.com/sharepoint/v3/fields"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1177B4BE-B106-4A5F-9B8B-849CAD24B948}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="576ce185-3b2e-4f75-8b7c-efeb82226bea"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5FA61470-DD61-4999-8627-225AC049B66F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{947F1741-2986-4B63-8B5C-D0468C671233}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A1C5838C-81AB-4B9A-B282-4E4B57DAFB8B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FD45C59E-C13E-4B92-9551-AE1790848EFA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1243,45 +1289,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A1C5838C-81AB-4B9A-B282-4E4B57DAFB8B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{947F1741-2986-4B63-8B5C-D0468C671233}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5FA61470-DD61-4999-8627-225AC049B66F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1177B4BE-B106-4A5F-9B8B-849CAD24B948}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="576ce185-3b2e-4f75-8b7c-efeb82226bea"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>